<commit_message>
v2 terminada y para entregar
</commit_message>
<xml_diff>
--- a/docTemplates/XLSXTemplate.xlsx
+++ b/docTemplates/XLSXTemplate.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\personal\Zenttric\clinic\docTemplates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikolai\Desktop\Zenttric\clinic\docTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14497EC9-2952-4507-A28B-834230EEE1F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C20F65-AD0D-4A04-9174-7CC18D7F1F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="header">Tabelle1!$A$1:$E$1</definedName>
-    <definedName name="Paciente">Tabelle1!$A$2:$E$2</definedName>
+    <definedName name="header">Tabelle1!$A$1:$I$1</definedName>
+    <definedName name="Paciente">Tabelle1!$A$2:$I$2</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>nombre</t>
   </si>
@@ -59,6 +59,30 @@
   </si>
   <si>
     <t>${fechaNacimiento}</t>
+  </si>
+  <si>
+    <t>tipoDocumento</t>
+  </si>
+  <si>
+    <t>numeroDocumento</t>
+  </si>
+  <si>
+    <t>telefono</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>${numeroDocumento}</t>
+  </si>
+  <si>
+    <t>${telefono}</t>
+  </si>
+  <si>
+    <t>${email}</t>
+  </si>
+  <si>
+    <t>${tipoDocumento}</t>
   </si>
 </sst>
 </file>
@@ -102,10 +126,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -386,49 +413,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.453125" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" customWidth="1"/>
-    <col min="3" max="3" width="14.90625" customWidth="1"/>
-    <col min="4" max="4" width="27" customWidth="1"/>
-    <col min="5" max="5" width="17.6328125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>8</v>
       </c>
+      <c r="F1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
+      <c r="F2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>